<commit_message>
Modified file Functional_TestSuite.xlsx with new Login TCs, added new file login-functionality-bugs.md and created a bug report for login functionality
</commit_message>
<xml_diff>
--- a/OrangeHRM/Functional_TestSuite.xlsx
+++ b/OrangeHRM/Functional_TestSuite.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="5"/>
+    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Test Suite Overview" sheetId="1" r:id="rId1"/>
@@ -19,11 +19,11 @@
     <sheet name="Login" sheetId="2" r:id="rId2"/>
     <sheet name="User Management" sheetId="14" r:id="rId10"/>
     <sheet name="PIM" sheetId="7" r:id="rId11"/>
-    <sheet name="Leave" sheetId="8" r:id="rId12"/>
+    <sheet name="Leave" sheetId="15" r:id="rId3"/>
     <sheet name="Time" sheetId="10" r:id="rId13"/>
     <sheet name="Performance" sheetId="11" r:id="rId14"/>
     <sheet name="Dashboard" sheetId="12" r:id="rId15"/>
-    <sheet name="Logout" sheetId="13" r:id="rId16"/>
+    <sheet name="Logout" sheetId="16" r:id="rId18"/>
     <sheet name="Recruitment" sheetId="9" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -388,12 +388,361 @@
   <si>
     <t>Pass</t>
   </si>
+  <si>
+    <t>TC-UM-002</t>
+  </si>
+  <si>
+    <t>Verify employee cannot access admin module</t>
+  </si>
+  <si>
+    <t>Employee logged in</t>
+  </si>
+  <si>
+    <t>1. Login as employee
+2. Try opening Admin module</t>
+  </si>
+  <si>
+    <t>Admin module is not available</t>
+  </si>
+  <si>
+    <t>TC-L-001</t>
+  </si>
+  <si>
+    <t>Verify Employee can apply for leave</t>
+  </si>
+  <si>
+    <t>1. Navigate to Leave</t>
+  </si>
+  <si>
+    <t>1. Navigate to Leave
+2. Select leave type
+3. Select dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to Leave
+2. Select leave type
+3. Select dates
+4. </t>
+  </si>
+  <si>
+    <t>1. Navigate to Leave Tab
+2. Select leave type
+3. Select dates from - to
+4. Click 'Apply' button</t>
+  </si>
+  <si>
+    <t>Leave: CAN - Vacation</t>
+  </si>
+  <si>
+    <t>Leave request should be submitted successfully.</t>
+  </si>
+  <si>
+    <t>Leave request should be submitted successfully.
+Leave request is displayed in 'My Leave' tab</t>
+  </si>
+  <si>
+    <t>TC-L-002</t>
+  </si>
+  <si>
+    <t>Verify Admin can approve leave request</t>
+  </si>
+  <si>
+    <t>Admin logged in
+Leave request exists</t>
+  </si>
+  <si>
+    <t>1. Admin logged in
+2. Leave request exists</t>
+  </si>
+  <si>
+    <t>1. Havigate to Leave Tab
+2. Click on 'Approve' button</t>
+  </si>
+  <si>
+    <t>Leave request should change to Approved</t>
+  </si>
+  <si>
+    <t>Leave request status should be changed to Scheduled</t>
+  </si>
+  <si>
+    <t>TC-LEAVE-001</t>
+  </si>
+  <si>
+    <t>TC-LEAVE-002</t>
+  </si>
+  <si>
+    <t>TC-LOGOUT-001</t>
+  </si>
+  <si>
+    <t>Verify user can logout successfully</t>
+  </si>
+  <si>
+    <t>User logged in</t>
+  </si>
+  <si>
+    <t>1. Click profile icon
+2. Click 'Logout' button</t>
+  </si>
+  <si>
+    <t>User should be redirected to login page</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>TC-LOGIN</t>
+  </si>
+  <si>
+    <t>Verify new admin can login with valid credentials</t>
+  </si>
+  <si>
+    <t>New Admin account created</t>
+  </si>
+  <si>
+    <t>Username: Admin</t>
+  </si>
+  <si>
+    <t>Password: admin123</t>
+  </si>
+  <si>
+    <t>Username: IamNewAdmin
+Password: IamNewAdmin123</t>
+  </si>
+  <si>
+    <t>User logged in successfully</t>
+  </si>
+  <si>
+    <t>TC-UM-003</t>
+  </si>
+  <si>
+    <t>Ts002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify </t>
+  </si>
+  <si>
+    <t>Admin can login with valid credentials</t>
+  </si>
+  <si>
+    <t>Employee can login with valid credetials</t>
+  </si>
+  <si>
+    <t>Error message for invalid password</t>
+  </si>
+  <si>
+    <t>New admin can login with valid credentials</t>
+  </si>
+  <si>
+    <t>Admin can add a new employee</t>
+  </si>
+  <si>
+    <t>Employee cannot access admin module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employee attempts to access Admin module by URL directly </t>
+  </si>
+  <si>
+    <t>1. Login as employee
+2. Copy the Admin module URL</t>
+  </si>
+  <si>
+    <t>1. Login as employee
+2. Copy the Admin module URL
+3. Paste the Admin module URL directly into browser
+4. Press Enter</t>
+  </si>
+  <si>
+    <t>Access is denied. User is redirected to an authorized page or receives an 'Access Denied' message.</t>
+  </si>
+  <si>
+    <t>Username: IamEmployeeJohn</t>
+  </si>
+  <si>
+    <t>Password: IAmEmployee123</t>
+  </si>
+  <si>
+    <t>1. Login as employee
+2. Copy the Admin module URL - https://opensource-demo.orangehrmlive.com/web/index.php/admin/viewSystemUsers
+3. Paste the Admin module URL directly into browser
+4. Press Enter</t>
+  </si>
+  <si>
+    <t>Access is denied. User receives 'Credential Required' message.</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-004</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User </t>
+  </si>
+  <si>
+    <t>User resets password using registered emeail</t>
+  </si>
+  <si>
+    <t>1. Open login page: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+2. Enter valid username
+3. Click 'Reset Password' link</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out</t>
+  </si>
+  <si>
+    <t>1. Open login page: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+2. Enter valid username
+3. Click 'Reset Password' link
+4. Enter the username
+5. Click 'Reset Password' button</t>
+  </si>
+  <si>
+    <t>The Reset password link is send successfully</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>BUG-LOGIN-001</t>
+  </si>
+  <si>
+    <t>BUG-LOGIN-005</t>
+  </si>
+  <si>
+    <t>BUG-001-LOGIN</t>
+  </si>
+  <si>
+    <t>User resets password using registered email</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>504 while reseting a password</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out appears after user resets password using registered email</t>
+  </si>
+  <si>
+    <t>504 after reseting a password</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out appears after user clicks 'Reset password' button</t>
+  </si>
+  <si>
+    <t>2. Enter valid username</t>
+  </si>
+  <si>
+    <t>3. Click 'Reset Password' link</t>
+  </si>
+  <si>
+    <t>4. Enter the username</t>
+  </si>
+  <si>
+    <t>5. Click 'Reset Password' button</t>
+  </si>
+  <si>
+    <t>The Reset password link is send to the user email successfully</t>
+  </si>
+  <si>
+    <t>1. Open login page: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+2. Enter valid username
+3. Click 'Reset Password' link
+4. Enter the existing username
+5. Click 'Reset Password' button</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out accurs after reseting a password</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out accurs after clicking 'Reset Password' on OrangeHRM login</t>
+  </si>
+  <si>
+    <t>After submitting the 'Reset Password' request in the OrangeHRM demo site, the system returns a 504 Gateway Time-out error.</t>
+  </si>
+  <si>
+    <t>1. Open login page: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+2. Enter a valid username
+3. Click 'Reset Password' link
+4. Enter the existing username
+5. Click 'Reset Password' button</t>
+  </si>
+  <si>
+    <t>Password reset request should complete successfuly.
+User should see confirmation message.
+No server error (504) should occur.</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out error massage occurs</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Google Chrome
+Version 149.0.7827.104</t>
+  </si>
+  <si>
+    <t>Password reset request should complete successfuly.
+User should see confirmation message - 'Reset Password link sent successfully'
+No server error (504) should occur.</t>
+  </si>
+  <si>
+    <t>When a user attempts to reset their password using the 'Forgot Password' fuctionality, the system returns a 504 Gateway Time-out error.</t>
+  </si>
+  <si>
+    <t>1. Open login page: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+2. Enter a valid username
+3. Click 'Forgot your password?' link
+4. Enter the existing username
+5. Click 'Reset Password' button</t>
+  </si>
+  <si>
+    <t>504 Gateway Time-out error occurs</t>
+  </si>
+  <si>
+    <t>URL: Google Chrome
+Version 149.0.7827.104</t>
+  </si>
+  <si>
+    <t>URL: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+Browser: Google Chrome, Version 149.0.7827.104</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>Intermittent</t>
+  </si>
+  <si>
+    <t>URL: https://opensource-demo.orangehrmlive.com/web/index.php/auth/login
+Browser: Google Chrome, Version 149.0.7827.104</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Valid user account exists in the system</t>
+  </si>
+  <si>
+    <t>1. Open login page
+2. Enter a valid username
+3. Click 'Forgot your password?' link
+4. Enter the existing username
+5. Click 'Reset Password' button</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -401,8 +750,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <color rgb="FFFF0000"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -459,6 +815,21 @@
         <fgColor rgb="FF7F7F7F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8FAADB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB3C6E7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -472,7 +843,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="2" applyFill="1" xfId="0"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="3" applyFill="1" xfId="0"/>
@@ -490,6 +861,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="11" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="12" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="13" applyFill="1" xfId="0"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="14" applyFill="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -917,7 +1292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
@@ -925,10 +1300,104 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0" defaultColWidth="8.609375"/>
+  <cols>
+    <col min="1" max="1" width="15.19921875" customWidth="1"/>
+    <col min="2" max="2" width="11.296875" customWidth="1"/>
+    <col min="3" max="3" width="22.59765625" customWidth="1"/>
+    <col min="4" max="4" width="15.87109375" customWidth="1"/>
+    <col min="5" max="5" width="19.7734375" customWidth="1"/>
+    <col min="6" max="6" width="19.234375" customWidth="1"/>
+    <col min="7" max="7" width="20.17578125" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.76171875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" ht="28.5">
+      <c r="A2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J2" t="s">
+        <v>134</v>
+      </c>
+      <c r="K2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4">
+      <c r="C4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -995,7 +1464,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>58</v>
+        <v>146</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>59</v>
@@ -1027,7 +1496,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>97</v>
+        <v>147</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>95</v>
@@ -1059,7 +1528,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>79</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
         <v>80</v>
@@ -1082,6 +1551,200 @@
       <c r="K4" t="s">
         <v>85</v>
       </c>
+    </row>
+    <row r="5" ht="123">
+      <c r="A5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" ht="177">
+      <c r="A6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="J6" t="s">
+        <v>67</v>
+      </c>
+      <c r="K6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0" defaultColWidth="8.609375"/>
+  <cols>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.296875" customWidth="1"/>
+    <col min="3" max="3" width="22.59765625" customWidth="1"/>
+    <col min="4" max="4" width="15.87109375" customWidth="1"/>
+    <col min="5" max="5" width="19.7734375" customWidth="1"/>
+    <col min="6" max="6" width="19.234375" customWidth="1"/>
+    <col min="7" max="7" width="20.17578125" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.76171875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" ht="82.5">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" ht="55.5">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1128,8 +1791,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="2" max="2" width="10.35546875" customWidth="1"/>
-    <col min="4" max="4" width="20.17578125" customWidth="1"/>
+    <col min="2" max="2" width="14.2578125" customWidth="1"/>
+    <col min="3" max="3" width="7.3984375" customWidth="1"/>
+    <col min="4" max="4" width="9.68359375" customWidth="1"/>
+    <col min="5" max="5" width="27.57421875" customWidth="1"/>
+    <col min="6" max="6" width="16.54296875" customWidth="1"/>
+    <col min="7" max="7" width="15.6015625" customWidth="1"/>
+    <col min="8" max="8" width="20.71484375" customWidth="1"/>
+    <col min="9" max="9" width="17.08203125" customWidth="1"/>
+    <col min="10" max="10" width="19.7734375" customWidth="1"/>
+    <col min="11" max="11" width="11.296875" customWidth="1"/>
+    <col min="12" max="12" width="10.22265625" customWidth="1"/>
+    <col min="13" max="13" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1137,19 +1810,81 @@
         <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="I1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2" ht="123">
+      <c r="A2" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M2" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1248,7 +1983,7 @@
         <v>34</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>87</v>
+        <v>150</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>88</v>
@@ -1272,18 +2007,69 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3">
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-    </row>
-    <row r="4">
-      <c r="C4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+    <row r="3" ht="55.5">
+      <c r="A3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" ht="150">
+      <c r="A4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" t="s">
+        <v>68</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1296,12 +2082,4 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>